<commit_message>
take the same name for Kongress
</commit_message>
<xml_diff>
--- a/data/tek_data/GHD_profile.xlsx
+++ b/data/tek_data/GHD_profile.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27328"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9F96CC3-A08D-4CE8-B44B-9B2087628A59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C67FEC4-DAA4-4275-A6F3-36495A4335FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1170" yWindow="2655" windowWidth="21600" windowHeight="11280" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SIA2024" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
-    <author>作者</author>
+    <author>Autor</author>
   </authors>
   <commentList>
     <comment ref="C23" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000001000000}">
@@ -36,7 +36,7 @@
             <rFont val="Segoe UI"/>
             <family val="2"/>
           </rPr>
-          <t>作者:</t>
+          <t>Autor:</t>
         </r>
         <r>
           <rPr>
@@ -60,7 +60,7 @@
             <rFont val="Segoe UI"/>
             <family val="2"/>
           </rPr>
-          <t>作者:</t>
+          <t>Autor:</t>
         </r>
         <r>
           <rPr>
@@ -84,7 +84,7 @@
             <rFont val="Segoe UI"/>
             <family val="2"/>
           </rPr>
-          <t>作者:</t>
+          <t>Autor:</t>
         </r>
         <r>
           <rPr>
@@ -543,9 +543,6 @@
     <t>Bühne (Theater und Veranstaltungsbauten)</t>
   </si>
   <si>
-    <t>Messe/Kongress</t>
-  </si>
-  <si>
     <t>Ausstellungsräume und Museum mit konservatorischen Anforderungen</t>
   </si>
   <si>
@@ -611,17 +608,20 @@
   <si>
     <t>Bettenzimmer</t>
     <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Messe / Kongress</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -629,14 +629,14 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -655,7 +655,7 @@
     </font>
     <font>
       <sz val="9"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -710,7 +710,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -989,30 +989,30 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:T45"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="34.44140625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="19.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.6640625" customWidth="1"/>
-    <col min="5" max="6" width="82.109375" customWidth="1"/>
-    <col min="7" max="7" width="17.109375" customWidth="1"/>
-    <col min="8" max="8" width="14.88671875" customWidth="1"/>
-    <col min="9" max="9" width="22.33203125" customWidth="1"/>
-    <col min="10" max="10" width="86.33203125" customWidth="1"/>
-    <col min="11" max="11" width="28.33203125" customWidth="1"/>
+    <col min="1" max="1" width="34.42578125" style="2" customWidth="1"/>
+    <col min="2" max="2" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.7109375" customWidth="1"/>
+    <col min="5" max="6" width="82.140625" customWidth="1"/>
+    <col min="7" max="7" width="17.140625" customWidth="1"/>
+    <col min="8" max="8" width="14.85546875" customWidth="1"/>
+    <col min="9" max="9" width="22.28515625" customWidth="1"/>
+    <col min="10" max="10" width="86.28515625" customWidth="1"/>
+    <col min="11" max="11" width="28.28515625" customWidth="1"/>
     <col min="12" max="12" width="28" customWidth="1"/>
-    <col min="13" max="13" width="22.6640625" customWidth="1"/>
-    <col min="14" max="14" width="23.5546875" customWidth="1"/>
-    <col min="15" max="15" width="15.109375" customWidth="1"/>
-    <col min="16" max="16" width="18.44140625" customWidth="1"/>
+    <col min="13" max="13" width="22.7109375" customWidth="1"/>
+    <col min="14" max="14" width="23.5703125" customWidth="1"/>
+    <col min="15" max="15" width="15.140625" customWidth="1"/>
+    <col min="16" max="16" width="18.42578125" customWidth="1"/>
     <col min="17" max="17" width="15" customWidth="1"/>
-    <col min="18" max="18" width="28.6640625" customWidth="1"/>
-    <col min="19" max="19" width="23.6640625" customWidth="1"/>
-    <col min="20" max="20" width="27.33203125" customWidth="1"/>
+    <col min="18" max="18" width="28.7109375" customWidth="1"/>
+    <col min="19" max="19" width="23.7109375" customWidth="1"/>
+    <col min="20" max="20" width="27.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20" s="4" customFormat="1">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1074,7 +1074,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:20">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -1136,7 +1136,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:20">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -1198,7 +1198,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:20">
       <c r="A4" s="2" t="s">
         <v>15</v>
       </c>
@@ -1260,7 +1260,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:20">
       <c r="A5" s="2" t="s">
         <v>19</v>
       </c>
@@ -1322,7 +1322,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:20">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -1384,7 +1384,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:20">
       <c r="A7" s="2" t="s">
         <v>21</v>
       </c>
@@ -1446,7 +1446,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:20">
       <c r="A8" s="2" t="s">
         <v>22</v>
       </c>
@@ -1508,7 +1508,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:20">
       <c r="A9" s="2" t="s">
         <v>23</v>
       </c>
@@ -1570,7 +1570,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:20">
       <c r="A10" s="2" t="s">
         <v>24</v>
       </c>
@@ -1632,7 +1632,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:20">
       <c r="A11" s="2" t="s">
         <v>25</v>
       </c>
@@ -1694,7 +1694,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:20">
       <c r="A12" s="2" t="s">
         <v>26</v>
       </c>
@@ -1756,7 +1756,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:20">
       <c r="A13" s="2" t="s">
         <v>27</v>
       </c>
@@ -1818,7 +1818,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:20">
       <c r="A14" s="2" t="s">
         <v>28</v>
       </c>
@@ -1880,7 +1880,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:20">
       <c r="A15" s="2" t="s">
         <v>29</v>
       </c>
@@ -1942,7 +1942,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:20">
       <c r="A16" s="2" t="s">
         <v>30</v>
       </c>
@@ -2004,7 +2004,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:20">
       <c r="A17" s="2" t="s">
         <v>31</v>
       </c>
@@ -2066,7 +2066,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:20">
       <c r="A18" s="2" t="s">
         <v>32</v>
       </c>
@@ -2128,7 +2128,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:20">
       <c r="A19" s="2" t="s">
         <v>33</v>
       </c>
@@ -2190,7 +2190,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:20">
       <c r="A20" s="2" t="s">
         <v>34</v>
       </c>
@@ -2252,7 +2252,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:20">
       <c r="A21" s="2" t="s">
         <v>35</v>
       </c>
@@ -2314,7 +2314,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:20">
       <c r="A22" s="2" t="s">
         <v>36</v>
       </c>
@@ -2376,7 +2376,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:20">
       <c r="A23" s="2" t="s">
         <v>65</v>
       </c>
@@ -2438,7 +2438,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:20">
       <c r="A24" s="2" t="s">
         <v>94</v>
       </c>
@@ -2500,7 +2500,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:20">
       <c r="A25" s="2" t="s">
         <v>37</v>
       </c>
@@ -2562,7 +2562,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="26" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:20">
       <c r="A26" s="2" t="s">
         <v>38</v>
       </c>
@@ -2624,7 +2624,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:20">
       <c r="A27" s="2" t="s">
         <v>39</v>
       </c>
@@ -2686,7 +2686,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="28" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:20">
       <c r="A28" s="2" t="s">
         <v>40</v>
       </c>
@@ -2748,7 +2748,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="29" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:20">
       <c r="A29" s="2" t="s">
         <v>41</v>
       </c>
@@ -2810,7 +2810,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="30" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:20">
       <c r="A30" s="2" t="s">
         <v>42</v>
       </c>
@@ -2872,7 +2872,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="31" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:20">
       <c r="A31" s="2" t="s">
         <v>43</v>
       </c>
@@ -2934,7 +2934,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:20">
       <c r="A32" s="2" t="s">
         <v>44</v>
       </c>
@@ -2996,7 +2996,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:20">
       <c r="A33" s="2" t="s">
         <v>45</v>
       </c>
@@ -3058,7 +3058,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:20">
       <c r="A34" s="2" t="s">
         <v>46</v>
       </c>
@@ -3120,7 +3120,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="35" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:20">
       <c r="A35" s="2" t="s">
         <v>47</v>
       </c>
@@ -3182,7 +3182,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="36" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:20">
       <c r="A36" s="2" t="s">
         <v>48</v>
       </c>
@@ -3244,7 +3244,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="37" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:20">
       <c r="A37" s="2" t="s">
         <v>49</v>
       </c>
@@ -3300,7 +3300,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:20">
       <c r="A38" s="2" t="s">
         <v>74</v>
       </c>
@@ -3356,7 +3356,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:20">
       <c r="A39" s="2" t="s">
         <v>50</v>
       </c>
@@ -3412,7 +3412,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:20">
       <c r="A40" s="2" t="s">
         <v>75</v>
       </c>
@@ -3468,7 +3468,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:20">
       <c r="A41" s="2" t="s">
         <v>51</v>
       </c>
@@ -3524,7 +3524,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:20">
       <c r="A42" s="2" t="s">
         <v>52</v>
       </c>
@@ -3577,7 +3577,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:20">
       <c r="A43" s="2" t="s">
         <v>53</v>
       </c>
@@ -3636,7 +3636,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:20">
       <c r="A44" s="2" t="s">
         <v>54</v>
       </c>
@@ -3695,7 +3695,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:20">
       <c r="A45" s="2" t="s">
         <v>55</v>
       </c>
@@ -3764,23 +3764,23 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:U44"/>
-  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
-    <col min="2" max="2" width="41.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="41.5703125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="29" customWidth="1"/>
     <col min="4" max="4" width="17" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="28.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="28.7109375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="28" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.44140625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="35.88671875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="27.44140625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="26.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="35.85546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="27.42578125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="26.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:21" s="4" customFormat="1">
       <c r="A1" s="4" t="s">
         <v>109</v>
       </c>
@@ -3832,7 +3832,7 @@
       <c r="T1" s="5"/>
       <c r="U1" s="5"/>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:21">
       <c r="A2">
         <v>1</v>
       </c>
@@ -3882,12 +3882,12 @@
         <v>7.1</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:21">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C3" t="s">
         <v>20</v>
@@ -3932,7 +3932,7 @@
         <v>7.1</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:21">
       <c r="A4">
         <v>3</v>
       </c>
@@ -3982,7 +3982,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:21">
       <c r="A5">
         <v>4</v>
       </c>
@@ -4032,7 +4032,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:21">
       <c r="A6">
         <v>5</v>
       </c>
@@ -4082,7 +4082,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:21">
       <c r="A7">
         <v>6</v>
       </c>
@@ -4132,12 +4132,12 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:21">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C8" t="s">
         <v>30</v>
@@ -4182,7 +4182,7 @@
         <v>-10</v>
       </c>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:21">
       <c r="A9">
         <v>8</v>
       </c>
@@ -4232,7 +4232,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:21">
       <c r="A10">
         <v>9</v>
       </c>
@@ -4282,12 +4282,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:21">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C11" t="s">
         <v>40</v>
@@ -4332,7 +4332,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:21">
       <c r="A12">
         <v>11</v>
       </c>
@@ -4382,7 +4382,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:21">
       <c r="A13">
         <v>12</v>
       </c>
@@ -4432,7 +4432,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:21">
       <c r="A14">
         <v>13</v>
       </c>
@@ -4482,12 +4482,12 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:21">
       <c r="A15">
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C15" s="8" t="s">
         <v>94</v>
@@ -4532,12 +4532,12 @@
         <v>300</v>
       </c>
     </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:21">
       <c r="A16">
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C16" t="s">
         <v>65</v>
@@ -4582,7 +4582,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:16">
       <c r="A17">
         <v>16</v>
       </c>
@@ -4632,12 +4632,12 @@
         <v>133</v>
       </c>
     </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:16">
       <c r="A18">
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C18" s="9" t="s">
         <v>37</v>
@@ -4682,7 +4682,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:16">
       <c r="A19">
         <v>18</v>
       </c>
@@ -4732,7 +4732,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:16">
       <c r="A20">
         <v>19</v>
       </c>
@@ -4782,7 +4782,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:16">
       <c r="A21">
         <v>20</v>
       </c>
@@ -4832,7 +4832,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:16">
       <c r="A22">
         <v>21</v>
       </c>
@@ -4882,7 +4882,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:16">
       <c r="A23" s="7" t="s">
         <v>139</v>
       </c>
@@ -4932,7 +4932,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:16">
       <c r="A24" s="7" t="s">
         <v>140</v>
       </c>
@@ -4982,12 +4982,12 @@
         <v>35</v>
       </c>
     </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:16">
       <c r="A25" s="6" t="s">
         <v>142</v>
       </c>
       <c r="B25" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C25" t="s">
         <v>44</v>
@@ -5032,7 +5032,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:16">
       <c r="A26">
         <v>23</v>
       </c>
@@ -5082,7 +5082,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:16">
       <c r="A27">
         <v>24</v>
       </c>
@@ -5132,7 +5132,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:16">
       <c r="A28">
         <v>25</v>
       </c>
@@ -5182,12 +5182,12 @@
         <v>133</v>
       </c>
     </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:16">
       <c r="A29">
         <v>26</v>
       </c>
       <c r="B29" t="s">
-        <v>146</v>
+        <v>168</v>
       </c>
       <c r="C29" t="s">
         <v>38</v>
@@ -5232,12 +5232,12 @@
         <v>2</v>
       </c>
     </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:16">
       <c r="A30">
         <v>27</v>
       </c>
       <c r="B30" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C30" t="s">
         <v>39</v>
@@ -5282,12 +5282,12 @@
         <v>133</v>
       </c>
     </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:16">
       <c r="A31">
         <v>28</v>
       </c>
       <c r="B31" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C31" t="s">
         <v>26</v>
@@ -5332,12 +5332,12 @@
         <v>133</v>
       </c>
     </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:16">
       <c r="A32">
         <v>29</v>
       </c>
       <c r="B32" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C32" t="s">
         <v>26</v>
@@ -5382,12 +5382,12 @@
         <v>133</v>
       </c>
     </row>
-    <row r="33" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:16">
       <c r="A33">
         <v>30</v>
       </c>
       <c r="B33" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C33" s="8" t="s">
         <v>26</v>
@@ -5432,12 +5432,12 @@
         <v>133</v>
       </c>
     </row>
-    <row r="34" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:16">
       <c r="A34">
         <v>31</v>
       </c>
       <c r="B34" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C34" t="s">
         <v>46</v>
@@ -5482,12 +5482,12 @@
         <v>133</v>
       </c>
     </row>
-    <row r="35" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:16">
       <c r="A35">
         <v>32</v>
       </c>
       <c r="B35" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C35" t="s">
         <v>52</v>
@@ -5532,12 +5532,12 @@
         <v>133</v>
       </c>
     </row>
-    <row r="36" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:16">
       <c r="A36">
         <v>33</v>
       </c>
       <c r="B36" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C36" t="s">
         <v>52</v>
@@ -5582,15 +5582,15 @@
         <v>133</v>
       </c>
     </row>
-    <row r="37" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:16">
       <c r="A37">
         <v>34</v>
       </c>
       <c r="B37" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C37" s="9" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D37">
         <v>11</v>
@@ -5632,7 +5632,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="38" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:16">
       <c r="A38">
         <v>35</v>
       </c>
@@ -5682,12 +5682,12 @@
         <v>2</v>
       </c>
     </row>
-    <row r="39" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:16">
       <c r="A39">
         <v>36</v>
       </c>
       <c r="B39" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C39" s="9" t="s">
         <v>28</v>
@@ -5732,12 +5732,12 @@
         <v>18</v>
       </c>
     </row>
-    <row r="40" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:16">
       <c r="A40">
         <v>37</v>
       </c>
       <c r="B40" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C40" t="s">
         <v>42</v>
@@ -5782,12 +5782,12 @@
         <v>7</v>
       </c>
     </row>
-    <row r="41" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:16">
       <c r="A41">
         <v>38</v>
       </c>
       <c r="B41" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C41" t="s">
         <v>41</v>
@@ -5832,12 +5832,12 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="42" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:16">
       <c r="A42">
         <v>39</v>
       </c>
       <c r="B42" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C42" t="s">
         <v>49</v>
@@ -5882,12 +5882,12 @@
         <v>133</v>
       </c>
     </row>
-    <row r="43" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:16">
       <c r="A43">
         <v>40</v>
       </c>
       <c r="B43" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C43" t="s">
         <v>42</v>
@@ -5932,12 +5932,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="44" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:16">
       <c r="A44">
         <v>41</v>
       </c>
       <c r="B44" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C44" t="s">
         <v>45</v>

</xml_diff>